<commit_message>
2026-08 age groups + adaptvie classifications
</commit_message>
<xml_diff>
--- a/local/agegroups/BARS-Results.xlsx
+++ b/local/agegroups/BARS-Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/Misc/usaw-owlcms/local/agegroups/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/agegroups/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE72CE0-8649-DE4B-85FC-92EF6114C99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6F72A0-2304-5E4B-9E50-02259E0B2882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1460" yWindow="500" windowWidth="39500" windowHeight="25100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1540" yWindow="600" windowWidth="39500" windowHeight="25100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="42">
   <si>
     <t>code</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>Masters</t>
+  </si>
+  <si>
+    <t>U11</t>
   </si>
 </sst>
 </file>
@@ -498,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W30"/>
+  <dimension ref="A1:W36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="2" width="23.5" customWidth="1"/>
@@ -546,7 +549,7 @@
     </row>
     <row r="2" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>38</v>
@@ -561,38 +564,42 @@
         <v>0</v>
       </c>
       <c r="F2" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G2" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2">
-        <v>36</v>
+      <c r="H2" s="2">
+        <v>30</v>
+      </c>
+      <c r="I2" s="2">
+        <v>33</v>
       </c>
       <c r="J2">
-        <v>40</v>
-      </c>
-      <c r="K2" s="1">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="K2">
+        <v>41</v>
       </c>
       <c r="L2" s="1">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M2" s="1">
+        <v>49</v>
+      </c>
+      <c r="N2" s="1">
         <v>53</v>
       </c>
-      <c r="N2" s="1">
-        <v>58</v>
-      </c>
       <c r="O2" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P2" s="1">
-        <v>999</v>
-      </c>
-      <c r="Q2" s="1"/>
+        <v>61</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>999</v>
+      </c>
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
@@ -601,7 +608,7 @@
     </row>
     <row r="3" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>38</v>
@@ -613,49 +620,54 @@
         <v>9</v>
       </c>
       <c r="E3" s="4">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F3" s="4">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G3" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="1"/>
+      <c r="H3" s="2">
+        <v>30</v>
+      </c>
+      <c r="I3" s="2">
+        <v>33</v>
+      </c>
       <c r="J3">
-        <v>40</v>
-      </c>
-      <c r="K3" s="1">
-        <v>44</v>
+        <v>37</v>
+      </c>
+      <c r="K3">
+        <v>41</v>
       </c>
       <c r="L3" s="1">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M3" s="1">
+        <v>49</v>
+      </c>
+      <c r="N3" s="1">
         <v>53</v>
       </c>
-      <c r="N3" s="1">
-        <v>58</v>
-      </c>
       <c r="O3" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P3" s="1">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="Q3" s="1">
         <v>999</v>
       </c>
-      <c r="R3" s="1"/>
       <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
       <c r="W3" s="1"/>
     </row>
     <row r="4" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>38</v>
@@ -667,91 +679,91 @@
         <v>9</v>
       </c>
       <c r="E4" s="4">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F4" s="4">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G4" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="H4" s="1"/>
-      <c r="K4" s="1">
-        <v>44</v>
+      <c r="K4">
+        <v>41</v>
       </c>
       <c r="L4" s="1">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M4" s="1">
+        <v>49</v>
+      </c>
+      <c r="N4" s="1">
         <v>53</v>
       </c>
-      <c r="N4" s="1">
-        <v>58</v>
-      </c>
       <c r="O4" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P4" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q4" s="1">
         <v>69</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="R4" s="1">
         <v>77</v>
       </c>
-      <c r="R4" s="1">
-        <v>999</v>
-      </c>
-      <c r="S4" s="1"/>
-      <c r="T4" s="1"/>
+      <c r="S4" s="1">
+        <v>999</v>
+      </c>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="4">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="F5" s="4">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="G5" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="H5" s="1"/>
-      <c r="K5" s="1"/>
       <c r="L5" s="1">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M5" s="1">
+        <v>49</v>
+      </c>
+      <c r="N5" s="1">
         <v>53</v>
       </c>
-      <c r="N5" s="1">
-        <v>58</v>
-      </c>
       <c r="O5" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P5" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q5" s="1">
         <v>69</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="R5" s="1">
         <v>77</v>
-      </c>
-      <c r="R5" s="1">
-        <v>86</v>
       </c>
       <c r="S5" s="1">
         <v>999</v>
@@ -763,7 +775,7 @@
     </row>
     <row r="6" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>40</v>
@@ -775,10 +787,10 @@
         <v>9</v>
       </c>
       <c r="E6" s="4">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F6" s="4">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="G6" s="5" t="b">
         <f>TRUE()</f>
@@ -786,38 +798,38 @@
       </c>
       <c r="H6" s="1"/>
       <c r="K6" s="1"/>
-      <c r="L6" s="1">
-        <v>48</v>
-      </c>
+      <c r="L6" s="1"/>
       <c r="M6" s="1">
+        <v>49</v>
+      </c>
+      <c r="N6" s="1">
         <v>53</v>
       </c>
-      <c r="N6" s="1">
-        <v>58</v>
-      </c>
       <c r="O6" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P6" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q6" s="1">
         <v>69</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="R6" s="1">
         <v>77</v>
       </c>
-      <c r="R6" s="1">
+      <c r="S6" s="1">
         <v>86</v>
       </c>
-      <c r="S6" s="1">
-        <v>999</v>
-      </c>
-      <c r="T6" s="1"/>
+      <c r="T6" s="1">
+        <v>999</v>
+      </c>
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>40</v>
@@ -829,10 +841,10 @@
         <v>9</v>
       </c>
       <c r="E7" s="4">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F7" s="4">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G7" s="5" t="b">
         <f>TRUE()</f>
@@ -840,38 +852,38 @@
       </c>
       <c r="H7" s="1"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="1">
-        <v>48</v>
-      </c>
+      <c r="L7" s="1"/>
       <c r="M7" s="1">
+        <v>49</v>
+      </c>
+      <c r="N7" s="1">
         <v>53</v>
       </c>
-      <c r="N7" s="1">
-        <v>58</v>
-      </c>
       <c r="O7" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P7" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q7" s="1">
         <v>69</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="R7" s="1">
         <v>77</v>
       </c>
-      <c r="R7" s="1">
+      <c r="S7" s="1">
         <v>86</v>
       </c>
-      <c r="S7" s="1">
-        <v>999</v>
-      </c>
-      <c r="T7" s="1"/>
+      <c r="T7" s="1">
+        <v>999</v>
+      </c>
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>40</v>
@@ -883,10 +895,10 @@
         <v>9</v>
       </c>
       <c r="E8" s="4">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F8" s="4">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G8" s="5" t="b">
         <f>TRUE()</f>
@@ -894,38 +906,38 @@
       </c>
       <c r="H8" s="1"/>
       <c r="K8" s="1"/>
-      <c r="L8" s="1">
-        <v>48</v>
-      </c>
+      <c r="L8" s="1"/>
       <c r="M8" s="1">
+        <v>49</v>
+      </c>
+      <c r="N8" s="1">
         <v>53</v>
       </c>
-      <c r="N8" s="1">
-        <v>58</v>
-      </c>
       <c r="O8" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P8" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q8" s="1">
         <v>69</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="R8" s="1">
         <v>77</v>
       </c>
-      <c r="R8" s="1">
+      <c r="S8" s="1">
         <v>86</v>
       </c>
-      <c r="S8" s="1">
-        <v>999</v>
-      </c>
-      <c r="T8" s="1"/>
+      <c r="T8" s="1">
+        <v>999</v>
+      </c>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
     </row>
     <row r="9" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>40</v>
@@ -937,10 +949,10 @@
         <v>9</v>
       </c>
       <c r="E9" s="4">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F9" s="4">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G9" s="5" t="b">
         <f>TRUE()</f>
@@ -948,38 +960,38 @@
       </c>
       <c r="H9" s="1"/>
       <c r="K9" s="1"/>
-      <c r="L9" s="1">
-        <v>48</v>
-      </c>
+      <c r="L9" s="1"/>
       <c r="M9" s="1">
+        <v>49</v>
+      </c>
+      <c r="N9" s="1">
         <v>53</v>
       </c>
-      <c r="N9" s="1">
-        <v>58</v>
-      </c>
       <c r="O9" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P9" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q9" s="1">
         <v>69</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="R9" s="1">
         <v>77</v>
       </c>
-      <c r="R9" s="1">
+      <c r="S9" s="1">
         <v>86</v>
       </c>
-      <c r="S9" s="1">
-        <v>999</v>
-      </c>
-      <c r="T9" s="1"/>
+      <c r="T9" s="1">
+        <v>999</v>
+      </c>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>40</v>
@@ -991,10 +1003,10 @@
         <v>9</v>
       </c>
       <c r="E10" s="4">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F10" s="4">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G10" s="5" t="b">
         <f>TRUE()</f>
@@ -1002,38 +1014,38 @@
       </c>
       <c r="H10" s="1"/>
       <c r="K10" s="1"/>
-      <c r="L10" s="1">
-        <v>48</v>
-      </c>
+      <c r="L10" s="1"/>
       <c r="M10" s="1">
+        <v>49</v>
+      </c>
+      <c r="N10" s="1">
         <v>53</v>
       </c>
-      <c r="N10" s="1">
-        <v>58</v>
-      </c>
       <c r="O10" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P10" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q10" s="1">
         <v>69</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="R10" s="1">
         <v>77</v>
       </c>
-      <c r="R10" s="1">
+      <c r="S10" s="1">
         <v>86</v>
       </c>
-      <c r="S10" s="1">
-        <v>999</v>
-      </c>
-      <c r="T10" s="1"/>
+      <c r="T10" s="1">
+        <v>999</v>
+      </c>
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>40</v>
@@ -1045,10 +1057,10 @@
         <v>9</v>
       </c>
       <c r="E11" s="4">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F11" s="4">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G11" s="5" t="b">
         <f>TRUE()</f>
@@ -1056,38 +1068,38 @@
       </c>
       <c r="H11" s="1"/>
       <c r="K11" s="1"/>
-      <c r="L11" s="1">
-        <v>48</v>
-      </c>
+      <c r="L11" s="1"/>
       <c r="M11" s="1">
+        <v>49</v>
+      </c>
+      <c r="N11" s="1">
         <v>53</v>
       </c>
-      <c r="N11" s="1">
-        <v>58</v>
-      </c>
       <c r="O11" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P11" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q11" s="1">
         <v>69</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="R11" s="1">
         <v>77</v>
       </c>
-      <c r="R11" s="1">
+      <c r="S11" s="1">
         <v>86</v>
       </c>
-      <c r="S11" s="1">
-        <v>999</v>
-      </c>
-      <c r="T11" s="1"/>
+      <c r="T11" s="1">
+        <v>999</v>
+      </c>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
     </row>
     <row r="12" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>40</v>
@@ -1099,10 +1111,10 @@
         <v>9</v>
       </c>
       <c r="E12" s="4">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F12" s="4">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G12" s="5" t="b">
         <f>TRUE()</f>
@@ -1110,38 +1122,38 @@
       </c>
       <c r="H12" s="1"/>
       <c r="K12" s="1"/>
-      <c r="L12" s="1">
-        <v>48</v>
-      </c>
+      <c r="L12" s="1"/>
       <c r="M12" s="1">
+        <v>49</v>
+      </c>
+      <c r="N12" s="1">
         <v>53</v>
       </c>
-      <c r="N12" s="1">
-        <v>58</v>
-      </c>
       <c r="O12" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P12" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q12" s="1">
         <v>69</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="R12" s="1">
         <v>77</v>
       </c>
-      <c r="R12" s="1">
+      <c r="S12" s="1">
         <v>86</v>
       </c>
-      <c r="S12" s="1">
-        <v>999</v>
-      </c>
-      <c r="T12" s="1"/>
+      <c r="T12" s="1">
+        <v>999</v>
+      </c>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>40</v>
@@ -1153,10 +1165,10 @@
         <v>9</v>
       </c>
       <c r="E13" s="4">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F13" s="4">
-        <v>999</v>
+        <v>74</v>
       </c>
       <c r="G13" s="5" t="b">
         <f>TRUE()</f>
@@ -1164,53 +1176,53 @@
       </c>
       <c r="H13" s="1"/>
       <c r="K13" s="1"/>
-      <c r="L13" s="1">
-        <v>48</v>
-      </c>
+      <c r="L13" s="1"/>
       <c r="M13" s="1">
+        <v>49</v>
+      </c>
+      <c r="N13" s="1">
         <v>53</v>
       </c>
-      <c r="N13" s="1">
-        <v>58</v>
-      </c>
       <c r="O13" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P13" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q13" s="1">
         <v>69</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="R13" s="1">
         <v>77</v>
       </c>
-      <c r="R13" s="1">
+      <c r="S13" s="1">
         <v>86</v>
       </c>
-      <c r="S13" s="1">
-        <v>999</v>
-      </c>
-      <c r="T13" s="1"/>
+      <c r="T13" s="1">
+        <v>999</v>
+      </c>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
       <c r="W13" s="1"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E14" s="4">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="F14" s="4">
-        <v>20</v>
+        <v>999</v>
       </c>
       <c r="G14" s="5" t="b">
         <f>TRUE()</f>
@@ -1218,53 +1230,53 @@
       </c>
       <c r="H14" s="1"/>
       <c r="K14" s="1"/>
-      <c r="L14" s="1">
-        <v>48</v>
-      </c>
+      <c r="L14" s="1"/>
       <c r="M14" s="1">
+        <v>49</v>
+      </c>
+      <c r="N14" s="1">
         <v>53</v>
       </c>
-      <c r="N14" s="1">
-        <v>58</v>
-      </c>
       <c r="O14" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P14" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q14" s="1">
         <v>69</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="R14" s="1">
         <v>77</v>
       </c>
-      <c r="R14" s="1">
+      <c r="S14" s="1">
         <v>86</v>
       </c>
-      <c r="S14" s="1">
-        <v>999</v>
-      </c>
-      <c r="T14" s="1"/>
+      <c r="T14" s="1">
+        <v>999</v>
+      </c>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
       <c r="W14" s="1"/>
     </row>
-    <row r="15" spans="1:23" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F15" s="4">
-        <v>999</v>
+        <v>20</v>
       </c>
       <c r="G15" s="5" t="b">
         <f>TRUE()</f>
@@ -1272,93 +1284,92 @@
       </c>
       <c r="H15" s="1"/>
       <c r="K15" s="1"/>
-      <c r="L15" s="1">
-        <v>48</v>
-      </c>
+      <c r="L15" s="1"/>
       <c r="M15" s="1">
+        <v>49</v>
+      </c>
+      <c r="N15" s="1">
         <v>53</v>
       </c>
-      <c r="N15" s="1">
-        <v>58</v>
-      </c>
       <c r="O15" s="1">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="P15" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q15" s="1">
         <v>69</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="R15" s="1">
         <v>77</v>
       </c>
-      <c r="R15" s="1">
+      <c r="S15" s="1">
         <v>86</v>
       </c>
-      <c r="S15" s="1">
-        <v>999</v>
-      </c>
-      <c r="T15" s="1"/>
+      <c r="T15" s="1">
+        <v>999</v>
+      </c>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
       <c r="W15" s="1"/>
     </row>
     <row r="16" spans="1:23" ht="15" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E16" s="4">
         <v>0</v>
       </c>
       <c r="F16" s="4">
-        <v>13</v>
+        <v>999</v>
       </c>
       <c r="G16" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H16" s="1">
-        <v>40</v>
-      </c>
-      <c r="I16">
-        <v>44</v>
-      </c>
-      <c r="J16">
-        <v>48</v>
-      </c>
-      <c r="K16" s="1">
-        <v>52</v>
-      </c>
-      <c r="L16" s="1">
-        <v>56</v>
-      </c>
+      <c r="H16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
       <c r="M16" s="1">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="N16" s="1">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="O16" s="1">
-        <v>999</v>
-      </c>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="1"/>
+        <v>57</v>
+      </c>
+      <c r="P16" s="1">
+        <v>61</v>
+      </c>
+      <c r="Q16" s="1">
+        <v>69</v>
+      </c>
+      <c r="R16" s="1">
+        <v>77</v>
+      </c>
+      <c r="S16" s="1">
+        <v>86</v>
+      </c>
+      <c r="T16" s="1">
+        <v>999</v>
+      </c>
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
+      <c r="W16" s="1"/>
     </row>
     <row r="17" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>38</v>
@@ -1370,36 +1381,41 @@
         <v>27</v>
       </c>
       <c r="E17" s="4">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F17" s="4">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G17" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H17" s="1"/>
+      <c r="H17" s="2">
+        <v>32</v>
+      </c>
+      <c r="I17" s="1">
+        <v>36</v>
+      </c>
       <c r="J17">
-        <v>48</v>
-      </c>
-      <c r="K17" s="1">
-        <v>52</v>
+        <v>40</v>
+      </c>
+      <c r="K17">
+        <v>45</v>
       </c>
       <c r="L17" s="1">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="M17" s="1">
+        <v>55</v>
+      </c>
+      <c r="N17" s="1">
         <v>60</v>
       </c>
-      <c r="N17" s="1">
+      <c r="O17" s="1">
         <v>65</v>
       </c>
-      <c r="O17" s="1">
-        <v>71</v>
-      </c>
       <c r="P17" s="1">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="Q17" s="1">
         <v>999</v>
@@ -1412,7 +1428,7 @@
     </row>
     <row r="18" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>38</v>
@@ -1424,91 +1440,99 @@
         <v>27</v>
       </c>
       <c r="E18" s="4">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F18" s="4">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G18" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H18" s="1"/>
-      <c r="K18" s="1"/>
+      <c r="H18" s="2">
+        <v>32</v>
+      </c>
+      <c r="I18" s="1">
+        <v>36</v>
+      </c>
+      <c r="J18">
+        <v>40</v>
+      </c>
+      <c r="K18">
+        <v>45</v>
+      </c>
       <c r="L18" s="1">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="M18" s="1">
+        <v>55</v>
+      </c>
+      <c r="N18" s="1">
         <v>60</v>
       </c>
-      <c r="N18" s="1">
+      <c r="O18" s="1">
         <v>65</v>
       </c>
-      <c r="O18" s="1">
-        <v>71</v>
-      </c>
       <c r="P18" s="1">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="Q18" s="1">
-        <v>88</v>
-      </c>
-      <c r="R18" s="1">
-        <v>94</v>
-      </c>
-      <c r="S18" s="1">
-        <v>999</v>
-      </c>
+        <v>999</v>
+      </c>
+      <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
       <c r="T18" s="1"/>
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
     </row>
     <row r="19" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="E19" s="4">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="F19" s="4">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="G19" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="1"/>
+      <c r="L19" s="1">
+        <v>50</v>
+      </c>
       <c r="M19" s="1">
+        <v>55</v>
+      </c>
+      <c r="N19" s="1">
         <v>60</v>
       </c>
-      <c r="N19" s="1">
+      <c r="O19" s="1">
         <v>65</v>
       </c>
-      <c r="O19" s="1">
-        <v>71</v>
-      </c>
       <c r="P19" s="1">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="Q19" s="1">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="R19" s="1">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="S19" s="1">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="T19" s="1">
         <v>999</v>
@@ -1518,50 +1542,50 @@
     </row>
     <row r="20" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="E20" s="4">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="F20" s="4">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="G20" s="5" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H20" s="1"/>
+      <c r="H20" s="2"/>
       <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
+      <c r="L20" s="2"/>
       <c r="M20" s="1">
+        <v>55</v>
+      </c>
+      <c r="N20" s="1">
         <v>60</v>
       </c>
-      <c r="N20" s="1">
+      <c r="O20" s="1">
         <v>65</v>
       </c>
-      <c r="O20" s="1">
-        <v>71</v>
-      </c>
       <c r="P20" s="1">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="Q20" s="1">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="R20" s="1">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="S20" s="1">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="T20" s="1">
         <v>999</v>
@@ -1571,7 +1595,7 @@
     </row>
     <row r="21" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>40</v>
@@ -1583,10 +1607,10 @@
         <v>27</v>
       </c>
       <c r="E21" s="4">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F21" s="4">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="G21" s="5" t="b">
         <f>TRUE()</f>
@@ -1602,16 +1626,16 @@
         <v>65</v>
       </c>
       <c r="O21" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P21" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q21" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R21" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S21" s="1">
         <v>110</v>
@@ -1624,7 +1648,7 @@
     </row>
     <row r="22" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>40</v>
@@ -1636,10 +1660,10 @@
         <v>27</v>
       </c>
       <c r="E22" s="4">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F22" s="4">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="G22" s="5" t="b">
         <f>TRUE()</f>
@@ -1655,16 +1679,16 @@
         <v>65</v>
       </c>
       <c r="O22" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P22" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q22" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R22" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S22" s="1">
         <v>110</v>
@@ -1677,7 +1701,7 @@
     </row>
     <row r="23" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>40</v>
@@ -1689,10 +1713,10 @@
         <v>27</v>
       </c>
       <c r="E23" s="4">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="F23" s="4">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="G23" s="5" t="b">
         <f>TRUE()</f>
@@ -1708,16 +1732,16 @@
         <v>65</v>
       </c>
       <c r="O23" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P23" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q23" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R23" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S23" s="1">
         <v>110</v>
@@ -1730,7 +1754,7 @@
     </row>
     <row r="24" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>40</v>
@@ -1742,10 +1766,10 @@
         <v>27</v>
       </c>
       <c r="E24" s="4">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F24" s="4">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="G24" s="5" t="b">
         <f>TRUE()</f>
@@ -1761,16 +1785,16 @@
         <v>65</v>
       </c>
       <c r="O24" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P24" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q24" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R24" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S24" s="1">
         <v>110</v>
@@ -1783,7 +1807,7 @@
     </row>
     <row r="25" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>40</v>
@@ -1795,10 +1819,10 @@
         <v>27</v>
       </c>
       <c r="E25" s="4">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="F25" s="4">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="G25" s="5" t="b">
         <f>TRUE()</f>
@@ -1814,16 +1838,16 @@
         <v>65</v>
       </c>
       <c r="O25" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P25" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q25" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R25" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S25" s="1">
         <v>110</v>
@@ -1836,7 +1860,7 @@
     </row>
     <row r="26" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>40</v>
@@ -1848,10 +1872,10 @@
         <v>27</v>
       </c>
       <c r="E26" s="4">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F26" s="4">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="G26" s="5" t="b">
         <f>TRUE()</f>
@@ -1867,16 +1891,16 @@
         <v>65</v>
       </c>
       <c r="O26" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P26" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q26" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R26" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S26" s="1">
         <v>110</v>
@@ -1889,7 +1913,7 @@
     </row>
     <row r="27" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>40</v>
@@ -1901,10 +1925,10 @@
         <v>27</v>
       </c>
       <c r="E27" s="4">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F27" s="4">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="G27" s="5" t="b">
         <f>TRUE()</f>
@@ -1920,16 +1944,16 @@
         <v>65</v>
       </c>
       <c r="O27" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P27" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q27" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R27" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S27" s="1">
         <v>110</v>
@@ -1941,8 +1965,8 @@
       <c r="V27" s="1"/>
     </row>
     <row r="28" spans="1:22" ht="15" x14ac:dyDescent="0.2">
-      <c r="A28" s="6" t="s">
-        <v>37</v>
+      <c r="A28" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>40</v>
@@ -1954,10 +1978,10 @@
         <v>27</v>
       </c>
       <c r="E28" s="4">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F28" s="4">
-        <v>999</v>
+        <v>74</v>
       </c>
       <c r="G28" s="5" t="b">
         <f>TRUE()</f>
@@ -1973,16 +1997,16 @@
         <v>65</v>
       </c>
       <c r="O28" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P28" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q28" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R28" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S28" s="1">
         <v>110</v>
@@ -1995,22 +2019,22 @@
     </row>
     <row r="29" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="E29" s="4">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="F29" s="4">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="G29" s="5" t="b">
         <f>TRUE()</f>
@@ -2026,16 +2050,16 @@
         <v>65</v>
       </c>
       <c r="O29" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P29" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q29" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R29" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S29" s="1">
         <v>110</v>
@@ -2047,20 +2071,20 @@
       <c r="V29" s="1"/>
     </row>
     <row r="30" spans="1:22" ht="15" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
-        <v>25</v>
+      <c r="A30" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>27</v>
       </c>
       <c r="E30" s="4">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F30" s="4">
         <v>999</v>
@@ -2079,16 +2103,16 @@
         <v>65</v>
       </c>
       <c r="O30" s="1">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P30" s="1">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="Q30" s="1">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="R30" s="1">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S30" s="1">
         <v>110</v>
@@ -2098,6 +2122,152 @@
       </c>
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
+    </row>
+    <row r="31" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="4">
+        <v>15</v>
+      </c>
+      <c r="F31" s="4">
+        <v>20</v>
+      </c>
+      <c r="G31" s="5" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1">
+        <v>60</v>
+      </c>
+      <c r="N31" s="1">
+        <v>65</v>
+      </c>
+      <c r="O31" s="1">
+        <v>70</v>
+      </c>
+      <c r="P31" s="1">
+        <v>75</v>
+      </c>
+      <c r="Q31" s="1">
+        <v>85</v>
+      </c>
+      <c r="R31" s="1">
+        <v>95</v>
+      </c>
+      <c r="S31" s="1">
+        <v>110</v>
+      </c>
+      <c r="T31" s="1">
+        <v>999</v>
+      </c>
+      <c r="U31" s="1"/>
+      <c r="V31" s="1"/>
+    </row>
+    <row r="32" spans="1:22" ht="15" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E32" s="4">
+        <v>0</v>
+      </c>
+      <c r="F32" s="4">
+        <v>999</v>
+      </c>
+      <c r="G32" s="5" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="H32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1">
+        <v>60</v>
+      </c>
+      <c r="N32" s="1">
+        <v>65</v>
+      </c>
+      <c r="O32" s="1">
+        <v>70</v>
+      </c>
+      <c r="P32" s="1">
+        <v>75</v>
+      </c>
+      <c r="Q32" s="1">
+        <v>85</v>
+      </c>
+      <c r="R32" s="1">
+        <v>95</v>
+      </c>
+      <c r="S32" s="1">
+        <v>110</v>
+      </c>
+      <c r="T32" s="1">
+        <v>999</v>
+      </c>
+      <c r="U32" s="1"/>
+      <c r="V32" s="1"/>
+    </row>
+    <row r="33" spans="13:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
+      <c r="T33" s="1"/>
+    </row>
+    <row r="34" spans="13:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
+      <c r="S34" s="1"/>
+      <c r="T34" s="1"/>
+    </row>
+    <row r="35" spans="13:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+      <c r="P35" s="1"/>
+      <c r="Q35" s="1"/>
+      <c r="R35" s="1"/>
+      <c r="S35" s="1"/>
+      <c r="T35" s="1"/>
+    </row>
+    <row r="36" spans="13:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1"/>
+      <c r="P36" s="1"/>
+      <c r="Q36" s="1"/>
+      <c r="R36" s="1"/>
+      <c r="S36" s="1"/>
+      <c r="T36" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>